<commit_message>
docs: add Sopyan back to team members and update Gantt chart
</commit_message>
<xml_diff>
--- a/project_management/Gantt_Chart_3_Minggu.xlsx
+++ b/project_management/Gantt_Chart_3_Minggu.xlsx
@@ -61,7 +61,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -88,8 +88,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0038A169"/>
-        <bgColor rgb="0038A169"/>
+        <fgColor rgb="00805AD5"/>
+        <bgColor rgb="00805AD5"/>
       </patternFill>
     </fill>
     <fill>
@@ -100,14 +100,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="0038A169"/>
+        <bgColor rgb="0038A169"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="003182CE"/>
         <bgColor rgb="003182CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00805AD5"/>
-        <bgColor rgb="00805AD5"/>
+        <fgColor rgb="00E53E3E"/>
+        <bgColor rgb="00E53E3E"/>
       </patternFill>
     </fill>
   </fills>
@@ -184,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -224,6 +230,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -591,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC22"/>
+  <dimension ref="A1:AC23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -635,7 +642,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sistem Informasi Komoditas Desa &amp; Keuangan Modern - Estimasi Jadwal Kerja 3 Minggu (Aldi &amp; Julia)</t>
+          <t>Sistem Informasi Komoditas Desa &amp; Keuangan Modern - Estimasi Jadwal Kerja 3 Minggu (Aldi, Julia, &amp; Sopyan)</t>
         </is>
       </c>
     </row>
@@ -820,7 +827,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Julia</t>
+          <t>Julia &amp; Sopyan</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -900,8 +907,8 @@
       </c>
       <c r="I7" s="14" t="n"/>
       <c r="J7" s="14" t="n"/>
-      <c r="K7" s="10" t="n"/>
-      <c r="L7" s="10" t="n"/>
+      <c r="K7" s="15" t="n"/>
+      <c r="L7" s="15" t="n"/>
       <c r="M7" s="14" t="n"/>
       <c r="N7" s="14" t="n"/>
       <c r="O7" s="14" t="n"/>
@@ -960,8 +967,8 @@
       <c r="I8" s="5" t="n"/>
       <c r="J8" s="5" t="n"/>
       <c r="K8" s="5" t="n"/>
-      <c r="L8" s="15" t="n"/>
-      <c r="M8" s="15" t="n"/>
+      <c r="L8" s="16" t="n"/>
+      <c r="M8" s="16" t="n"/>
       <c r="N8" s="5" t="n"/>
       <c r="O8" s="5" t="n"/>
       <c r="P8" s="5" t="n"/>
@@ -1020,8 +1027,8 @@
       <c r="J9" s="14" t="n"/>
       <c r="K9" s="14" t="n"/>
       <c r="L9" s="14" t="n"/>
-      <c r="M9" s="15" t="n"/>
-      <c r="N9" s="15" t="n"/>
+      <c r="M9" s="16" t="n"/>
+      <c r="N9" s="16" t="n"/>
       <c r="O9" s="14" t="n"/>
       <c r="P9" s="14" t="n"/>
       <c r="Q9" s="14" t="n"/>
@@ -1081,9 +1088,9 @@
       <c r="L10" s="5" t="n"/>
       <c r="M10" s="5" t="n"/>
       <c r="N10" s="5" t="n"/>
-      <c r="O10" s="15" t="n"/>
-      <c r="P10" s="15" t="n"/>
-      <c r="Q10" s="15" t="n"/>
+      <c r="O10" s="16" t="n"/>
+      <c r="P10" s="16" t="n"/>
+      <c r="Q10" s="16" t="n"/>
       <c r="R10" s="5" t="n"/>
       <c r="S10" s="5" t="n"/>
       <c r="T10" s="5" t="n"/>
@@ -1142,10 +1149,10 @@
       <c r="N11" s="14" t="n"/>
       <c r="O11" s="14" t="n"/>
       <c r="P11" s="14" t="n"/>
-      <c r="Q11" s="10" t="n"/>
-      <c r="R11" s="10" t="n"/>
-      <c r="S11" s="10" t="n"/>
-      <c r="T11" s="10" t="n"/>
+      <c r="Q11" s="15" t="n"/>
+      <c r="R11" s="15" t="n"/>
+      <c r="S11" s="15" t="n"/>
+      <c r="T11" s="15" t="n"/>
       <c r="U11" s="14" t="n"/>
       <c r="V11" s="14" t="n"/>
       <c r="W11" s="14" t="n"/>
@@ -1202,10 +1209,10 @@
       <c r="O12" s="5" t="n"/>
       <c r="P12" s="5" t="n"/>
       <c r="Q12" s="5" t="n"/>
-      <c r="R12" s="10" t="n"/>
-      <c r="S12" s="10" t="n"/>
-      <c r="T12" s="10" t="n"/>
-      <c r="U12" s="10" t="n"/>
+      <c r="R12" s="15" t="n"/>
+      <c r="S12" s="15" t="n"/>
+      <c r="T12" s="15" t="n"/>
+      <c r="U12" s="15" t="n"/>
       <c r="V12" s="5" t="n"/>
       <c r="W12" s="5" t="n"/>
       <c r="X12" s="5" t="n"/>
@@ -1263,9 +1270,9 @@
       <c r="Q13" s="14" t="n"/>
       <c r="R13" s="14" t="n"/>
       <c r="S13" s="14" t="n"/>
-      <c r="T13" s="10" t="n"/>
-      <c r="U13" s="10" t="n"/>
-      <c r="V13" s="10" t="n"/>
+      <c r="T13" s="15" t="n"/>
+      <c r="U13" s="15" t="n"/>
+      <c r="V13" s="15" t="n"/>
       <c r="W13" s="14" t="n"/>
       <c r="X13" s="14" t="n"/>
       <c r="Y13" s="14" t="n"/>
@@ -1292,7 +1299,7 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Aldi</t>
+          <t>Sopyan</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -1325,10 +1332,10 @@
       <c r="T14" s="5" t="n"/>
       <c r="U14" s="5" t="n"/>
       <c r="V14" s="5" t="n"/>
-      <c r="W14" s="15" t="n"/>
-      <c r="X14" s="15" t="n"/>
-      <c r="Y14" s="15" t="n"/>
-      <c r="Z14" s="15" t="n"/>
+      <c r="W14" s="17" t="n"/>
+      <c r="X14" s="17" t="n"/>
+      <c r="Y14" s="17" t="n"/>
+      <c r="Z14" s="17" t="n"/>
       <c r="AA14" s="5" t="n"/>
       <c r="AB14" s="5" t="n"/>
       <c r="AC14" s="5" t="n"/>
@@ -1386,10 +1393,10 @@
       <c r="V15" s="14" t="n"/>
       <c r="W15" s="14" t="n"/>
       <c r="X15" s="14" t="n"/>
-      <c r="Y15" s="15" t="n"/>
-      <c r="Z15" s="15" t="n"/>
-      <c r="AA15" s="15" t="n"/>
-      <c r="AB15" s="15" t="n"/>
+      <c r="Y15" s="16" t="n"/>
+      <c r="Z15" s="16" t="n"/>
+      <c r="AA15" s="16" t="n"/>
+      <c r="AB15" s="16" t="n"/>
       <c r="AC15" s="14" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -1446,9 +1453,9 @@
       <c r="W16" s="5" t="n"/>
       <c r="X16" s="5" t="n"/>
       <c r="Y16" s="5" t="n"/>
-      <c r="Z16" s="10" t="n"/>
-      <c r="AA16" s="10" t="n"/>
-      <c r="AB16" s="10" t="n"/>
+      <c r="Z16" s="15" t="n"/>
+      <c r="AA16" s="15" t="n"/>
+      <c r="AB16" s="15" t="n"/>
       <c r="AC16" s="5" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
@@ -1469,7 +1476,7 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Aldi &amp; Julia</t>
+          <t>Semua Tim</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
@@ -1506,40 +1513,48 @@
       <c r="X17" s="14" t="n"/>
       <c r="Y17" s="14" t="n"/>
       <c r="Z17" s="14" t="n"/>
-      <c r="AA17" s="16" t="n"/>
-      <c r="AB17" s="16" t="n"/>
-      <c r="AC17" s="16" t="n"/>
+      <c r="AA17" s="10" t="n"/>
+      <c r="AB17" s="10" t="n"/>
+      <c r="AC17" s="10" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="17" t="inlineStr">
+      <c r="B19" s="18" t="inlineStr">
         <is>
           <t>Legenda Penanggung Jawab:</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>Aldi Burung (Frontend / DB / Setup)</t>
         </is>
       </c>
-      <c r="C20" s="15" t="n"/>
+      <c r="C20" s="16" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="18" t="inlineStr">
+      <c r="B21" s="19" t="inlineStr">
         <is>
           <t>Julia (Analyst / Backend / QA)</t>
         </is>
       </c>
-      <c r="C21" s="10" t="n"/>
+      <c r="C21" s="15" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>Bersama (Handover &amp; Deployment)</t>
-        </is>
-      </c>
-      <c r="C22" s="16" t="n"/>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>Sopyan (Frontend / UI / UX)</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>Bersama (Gabungan Tim)</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="11">

</xml_diff>